<commit_message>
feat(T1.4): lectura del Excel y mapeo de filas con validación
- leerLibro: hojas Precio y Categorias; error de estructura aborta todo.
- mapearFila (puro): recompone MOD-MADERA-ANCHO-ALTO para puertas,
  2X<pulg> para marcos/piezas T y <cm>X<esp> para molduras; normaliza
  tildes (RAULÍ/RAULI); rechaza con motivo madera, tipo, ancho o alto
  desconocidos, precio inválido, neto ≠ costo × (1 + margen) y códigos
  repetidos.
- Validado contra el Excel real: 8.743 de 8.772 filas; 29 rechazos son
  errores del Excel (LLAG-O-2-A con alto 2,2 y marcos/piezas T de raulí
  con largo 2,0 en todas las filas).
- Fixtures: v2 escala costo y precio juntos.

Refs: REQ-STK-1.2, 1.4, DATA-MODEL §5
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e/fixtures/cotizador-mini-v2.xlsx
+++ b/e2e/fixtures/cotizador-mini-v2.xlsx
@@ -900,19 +900,19 @@
         <v>5</v>
       </c>
       <c r="I4">
-        <v>33750</v>
+        <v>37125</v>
       </c>
       <c r="J4">
-        <v>67500</v>
+        <v>74250</v>
       </c>
       <c r="K4">
-        <v>13500</v>
+        <v>14850</v>
       </c>
       <c r="L4">
-        <v>20250</v>
+        <v>22275</v>
       </c>
       <c r="M4">
-        <v>135000</v>
+        <v>148500</v>
       </c>
       <c r="N4">
         <v>0.2</v>
@@ -947,19 +947,19 @@
         <v>5</v>
       </c>
       <c r="I5">
-        <v>36250</v>
+        <v>39875</v>
       </c>
       <c r="J5">
-        <v>72500</v>
+        <v>79750</v>
       </c>
       <c r="K5">
-        <v>14500</v>
+        <v>15950</v>
       </c>
       <c r="L5">
-        <v>21750</v>
+        <v>23925</v>
       </c>
       <c r="M5">
-        <v>145000</v>
+        <v>159500</v>
       </c>
       <c r="N5">
         <v>0.2</v>
@@ -994,19 +994,19 @@
         <v>5</v>
       </c>
       <c r="I6">
-        <v>33750</v>
+        <v>37125</v>
       </c>
       <c r="J6">
-        <v>67500</v>
+        <v>74250</v>
       </c>
       <c r="K6">
-        <v>13500</v>
+        <v>14850</v>
       </c>
       <c r="L6">
-        <v>20250</v>
+        <v>22275</v>
       </c>
       <c r="M6">
-        <v>135000</v>
+        <v>148500</v>
       </c>
       <c r="N6">
         <v>0.2</v>
@@ -1041,19 +1041,19 @@
         <v>5</v>
       </c>
       <c r="I7">
-        <v>36250</v>
+        <v>39875</v>
       </c>
       <c r="J7">
-        <v>72500</v>
+        <v>79750</v>
       </c>
       <c r="K7">
-        <v>14500</v>
+        <v>15950</v>
       </c>
       <c r="L7">
-        <v>21750</v>
+        <v>23925</v>
       </c>
       <c r="M7">
-        <v>145000</v>
+        <v>159500</v>
       </c>
       <c r="N7">
         <v>0.2</v>
@@ -1088,19 +1088,19 @@
         <v>5</v>
       </c>
       <c r="I8">
-        <v>33750</v>
+        <v>37125</v>
       </c>
       <c r="J8">
-        <v>67500</v>
+        <v>74250</v>
       </c>
       <c r="K8">
-        <v>13500</v>
+        <v>14850</v>
       </c>
       <c r="L8">
-        <v>20250</v>
+        <v>22275</v>
       </c>
       <c r="M8">
-        <v>135000</v>
+        <v>148500</v>
       </c>
       <c r="N8">
         <v>0.2</v>
@@ -1135,19 +1135,19 @@
         <v>5</v>
       </c>
       <c r="I9">
-        <v>36250</v>
+        <v>39875</v>
       </c>
       <c r="J9">
-        <v>72500</v>
+        <v>79750</v>
       </c>
       <c r="K9">
-        <v>14500</v>
+        <v>15950</v>
       </c>
       <c r="L9">
-        <v>21750</v>
+        <v>23925</v>
       </c>
       <c r="M9">
-        <v>145000</v>
+        <v>159500</v>
       </c>
       <c r="N9">
         <v>0.2</v>
@@ -1182,19 +1182,19 @@
         <v>5</v>
       </c>
       <c r="I10">
-        <v>33750</v>
+        <v>37125</v>
       </c>
       <c r="J10">
-        <v>67500</v>
+        <v>74250</v>
       </c>
       <c r="K10">
-        <v>13500</v>
+        <v>14850</v>
       </c>
       <c r="L10">
-        <v>20250</v>
+        <v>22275</v>
       </c>
       <c r="M10">
-        <v>135000</v>
+        <v>148500</v>
       </c>
       <c r="N10">
         <v>0.2</v>
@@ -1229,19 +1229,19 @@
         <v>5</v>
       </c>
       <c r="I11">
-        <v>36250</v>
+        <v>39875</v>
       </c>
       <c r="J11">
-        <v>72500</v>
+        <v>79750</v>
       </c>
       <c r="K11">
-        <v>14500</v>
+        <v>15950</v>
       </c>
       <c r="L11">
-        <v>21750</v>
+        <v>23925</v>
       </c>
       <c r="M11">
-        <v>145000</v>
+        <v>159500</v>
       </c>
       <c r="N11">
         <v>0.2</v>
@@ -1276,19 +1276,19 @@
         <v>5</v>
       </c>
       <c r="I12">
-        <v>33750</v>
+        <v>37125</v>
       </c>
       <c r="J12">
-        <v>67500</v>
+        <v>74250</v>
       </c>
       <c r="K12">
-        <v>13500</v>
+        <v>14850</v>
       </c>
       <c r="L12">
-        <v>20250</v>
+        <v>22275</v>
       </c>
       <c r="M12">
-        <v>135000</v>
+        <v>148500</v>
       </c>
       <c r="N12">
         <v>0.2</v>
@@ -1323,19 +1323,19 @@
         <v>5</v>
       </c>
       <c r="I13">
-        <v>36250</v>
+        <v>39875</v>
       </c>
       <c r="J13">
-        <v>72500</v>
+        <v>79750</v>
       </c>
       <c r="K13">
-        <v>14500</v>
+        <v>15950</v>
       </c>
       <c r="L13">
-        <v>21750</v>
+        <v>23925</v>
       </c>
       <c r="M13">
-        <v>145000</v>
+        <v>159500</v>
       </c>
       <c r="N13">
         <v>0.2</v>
@@ -1370,19 +1370,19 @@
         <v>5</v>
       </c>
       <c r="I14">
-        <v>33750</v>
+        <v>37125</v>
       </c>
       <c r="J14">
-        <v>67500</v>
+        <v>74250</v>
       </c>
       <c r="K14">
-        <v>13500</v>
+        <v>14850</v>
       </c>
       <c r="L14">
-        <v>20250</v>
+        <v>22275</v>
       </c>
       <c r="M14">
-        <v>135000</v>
+        <v>148500</v>
       </c>
       <c r="N14">
         <v>0.3</v>
@@ -1417,19 +1417,19 @@
         <v>5</v>
       </c>
       <c r="I15">
-        <v>36250</v>
+        <v>39875</v>
       </c>
       <c r="J15">
-        <v>72500</v>
+        <v>79750</v>
       </c>
       <c r="K15">
-        <v>14500</v>
+        <v>15950</v>
       </c>
       <c r="L15">
-        <v>21750</v>
+        <v>23925</v>
       </c>
       <c r="M15">
-        <v>145000</v>
+        <v>159500</v>
       </c>
       <c r="N15">
         <v>0.3</v>
@@ -1464,19 +1464,19 @@
         <v>5</v>
       </c>
       <c r="I16">
-        <v>33750</v>
+        <v>37125</v>
       </c>
       <c r="J16">
-        <v>67500</v>
+        <v>74250</v>
       </c>
       <c r="K16">
-        <v>13500</v>
+        <v>14850</v>
       </c>
       <c r="L16">
-        <v>20250</v>
+        <v>22275</v>
       </c>
       <c r="M16">
-        <v>135000</v>
+        <v>148500</v>
       </c>
       <c r="N16">
         <v>0.3</v>
@@ -1511,19 +1511,19 @@
         <v>5</v>
       </c>
       <c r="I17">
-        <v>36250</v>
+        <v>39875</v>
       </c>
       <c r="J17">
-        <v>72500</v>
+        <v>79750</v>
       </c>
       <c r="K17">
-        <v>14500</v>
+        <v>15950</v>
       </c>
       <c r="L17">
-        <v>21750</v>
+        <v>23925</v>
       </c>
       <c r="M17">
-        <v>145000</v>
+        <v>159500</v>
       </c>
       <c r="N17">
         <v>0.3</v>
@@ -1558,19 +1558,19 @@
         <v>5</v>
       </c>
       <c r="I18">
-        <v>37500</v>
+        <v>41250</v>
       </c>
       <c r="J18">
-        <v>75000</v>
+        <v>82500</v>
       </c>
       <c r="K18">
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="L18">
-        <v>22500</v>
+        <v>24750</v>
       </c>
       <c r="M18">
-        <v>150000</v>
+        <v>165000</v>
       </c>
       <c r="N18">
         <v>0.3</v>
@@ -1605,19 +1605,19 @@
         <v>5</v>
       </c>
       <c r="I19">
-        <v>30000</v>
+        <v>33000</v>
       </c>
       <c r="J19">
-        <v>60000</v>
+        <v>66000</v>
       </c>
       <c r="K19">
-        <v>12000</v>
+        <v>13200</v>
       </c>
       <c r="L19">
-        <v>18000</v>
+        <v>19800</v>
       </c>
       <c r="M19">
-        <v>120000</v>
+        <v>132000</v>
       </c>
       <c r="N19">
         <v>0.2</v>
@@ -1652,19 +1652,19 @@
         <v>5</v>
       </c>
       <c r="I20">
-        <v>32500</v>
+        <v>35750</v>
       </c>
       <c r="J20">
-        <v>65000</v>
+        <v>71500</v>
       </c>
       <c r="K20">
-        <v>13000</v>
+        <v>14300</v>
       </c>
       <c r="L20">
-        <v>19500</v>
+        <v>21450</v>
       </c>
       <c r="M20">
-        <v>130000</v>
+        <v>143000</v>
       </c>
       <c r="N20">
         <v>0.2</v>
@@ -1699,19 +1699,19 @@
         <v>5</v>
       </c>
       <c r="I21">
-        <v>37500</v>
+        <v>41250</v>
       </c>
       <c r="J21">
-        <v>75000</v>
+        <v>82500</v>
       </c>
       <c r="K21">
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="L21">
-        <v>22500</v>
+        <v>24750</v>
       </c>
       <c r="M21">
-        <v>150000</v>
+        <v>165000</v>
       </c>
       <c r="N21">
         <v>0.2</v>
@@ -1746,19 +1746,19 @@
         <v>5</v>
       </c>
       <c r="I22">
-        <v>40000</v>
+        <v>44000</v>
       </c>
       <c r="J22">
-        <v>80000</v>
+        <v>88000</v>
       </c>
       <c r="K22">
-        <v>16000</v>
+        <v>17600</v>
       </c>
       <c r="L22">
-        <v>24000</v>
+        <v>26400</v>
       </c>
       <c r="M22">
-        <v>160000</v>
+        <v>176000</v>
       </c>
       <c r="N22">
         <v>0.2</v>
@@ -1793,19 +1793,19 @@
         <v>5</v>
       </c>
       <c r="I23">
-        <v>37500</v>
+        <v>41250</v>
       </c>
       <c r="J23">
-        <v>75000</v>
+        <v>82500</v>
       </c>
       <c r="K23">
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="L23">
-        <v>22500</v>
+        <v>24750</v>
       </c>
       <c r="M23">
-        <v>150000</v>
+        <v>165000</v>
       </c>
       <c r="N23">
         <v>0.2</v>
@@ -1840,19 +1840,19 @@
         <v>5</v>
       </c>
       <c r="I24">
-        <v>40000</v>
+        <v>44000</v>
       </c>
       <c r="J24">
-        <v>80000</v>
+        <v>88000</v>
       </c>
       <c r="K24">
-        <v>16000</v>
+        <v>17600</v>
       </c>
       <c r="L24">
-        <v>24000</v>
+        <v>26400</v>
       </c>
       <c r="M24">
-        <v>160000</v>
+        <v>176000</v>
       </c>
       <c r="N24">
         <v>0.2</v>
@@ -1887,19 +1887,19 @@
         <v>5</v>
       </c>
       <c r="I25">
-        <v>37500</v>
+        <v>41250</v>
       </c>
       <c r="J25">
-        <v>75000</v>
+        <v>82500</v>
       </c>
       <c r="K25">
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="L25">
-        <v>22500</v>
+        <v>24750</v>
       </c>
       <c r="M25">
-        <v>150000</v>
+        <v>165000</v>
       </c>
       <c r="N25">
         <v>0.2</v>
@@ -1934,19 +1934,19 @@
         <v>5</v>
       </c>
       <c r="I26">
-        <v>40000</v>
+        <v>44000</v>
       </c>
       <c r="J26">
-        <v>80000</v>
+        <v>88000</v>
       </c>
       <c r="K26">
-        <v>16000</v>
+        <v>17600</v>
       </c>
       <c r="L26">
-        <v>24000</v>
+        <v>26400</v>
       </c>
       <c r="M26">
-        <v>160000</v>
+        <v>176000</v>
       </c>
       <c r="N26">
         <v>0.2</v>
@@ -1981,19 +1981,19 @@
         <v>5</v>
       </c>
       <c r="I27">
-        <v>37500</v>
+        <v>41250</v>
       </c>
       <c r="J27">
-        <v>75000</v>
+        <v>82500</v>
       </c>
       <c r="K27">
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="L27">
-        <v>22500</v>
+        <v>24750</v>
       </c>
       <c r="M27">
-        <v>150000</v>
+        <v>165000</v>
       </c>
       <c r="N27">
         <v>0.2</v>
@@ -2028,19 +2028,19 @@
         <v>5</v>
       </c>
       <c r="I28">
-        <v>40000</v>
+        <v>44000</v>
       </c>
       <c r="J28">
-        <v>80000</v>
+        <v>88000</v>
       </c>
       <c r="K28">
-        <v>16000</v>
+        <v>17600</v>
       </c>
       <c r="L28">
-        <v>24000</v>
+        <v>26400</v>
       </c>
       <c r="M28">
-        <v>160000</v>
+        <v>176000</v>
       </c>
       <c r="N28">
         <v>0.2</v>
@@ -2075,19 +2075,19 @@
         <v>5</v>
       </c>
       <c r="I29">
-        <v>37500</v>
+        <v>41250</v>
       </c>
       <c r="J29">
-        <v>75000</v>
+        <v>82500</v>
       </c>
       <c r="K29">
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="L29">
-        <v>22500</v>
+        <v>24750</v>
       </c>
       <c r="M29">
-        <v>150000</v>
+        <v>165000</v>
       </c>
       <c r="N29">
         <v>0.2</v>
@@ -2122,19 +2122,19 @@
         <v>5</v>
       </c>
       <c r="I30">
-        <v>40000</v>
+        <v>44000</v>
       </c>
       <c r="J30">
-        <v>80000</v>
+        <v>88000</v>
       </c>
       <c r="K30">
-        <v>16000</v>
+        <v>17600</v>
       </c>
       <c r="L30">
-        <v>24000</v>
+        <v>26400</v>
       </c>
       <c r="M30">
-        <v>160000</v>
+        <v>176000</v>
       </c>
       <c r="N30">
         <v>0.2</v>
@@ -2169,19 +2169,19 @@
         <v>5</v>
       </c>
       <c r="I31">
-        <v>37500</v>
+        <v>41250</v>
       </c>
       <c r="J31">
-        <v>75000</v>
+        <v>82500</v>
       </c>
       <c r="K31">
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="L31">
-        <v>22500</v>
+        <v>24750</v>
       </c>
       <c r="M31">
-        <v>150000</v>
+        <v>165000</v>
       </c>
       <c r="N31">
         <v>0.3</v>
@@ -2216,19 +2216,19 @@
         <v>5</v>
       </c>
       <c r="I32">
-        <v>40000</v>
+        <v>44000</v>
       </c>
       <c r="J32">
-        <v>80000</v>
+        <v>88000</v>
       </c>
       <c r="K32">
-        <v>16000</v>
+        <v>17600</v>
       </c>
       <c r="L32">
-        <v>24000</v>
+        <v>26400</v>
       </c>
       <c r="M32">
-        <v>160000</v>
+        <v>176000</v>
       </c>
       <c r="N32">
         <v>0.3</v>
@@ -2263,19 +2263,19 @@
         <v>5</v>
       </c>
       <c r="I33">
-        <v>37500</v>
+        <v>41250</v>
       </c>
       <c r="J33">
-        <v>75000</v>
+        <v>82500</v>
       </c>
       <c r="K33">
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="L33">
-        <v>22500</v>
+        <v>24750</v>
       </c>
       <c r="M33">
-        <v>150000</v>
+        <v>165000</v>
       </c>
       <c r="N33">
         <v>0.3</v>
@@ -2310,19 +2310,19 @@
         <v>5</v>
       </c>
       <c r="I34">
-        <v>40000</v>
+        <v>44000</v>
       </c>
       <c r="J34">
-        <v>80000</v>
+        <v>88000</v>
       </c>
       <c r="K34">
-        <v>16000</v>
+        <v>17600</v>
       </c>
       <c r="L34">
-        <v>24000</v>
+        <v>26400</v>
       </c>
       <c r="M34">
-        <v>160000</v>
+        <v>176000</v>
       </c>
       <c r="N34">
         <v>0.3</v>
@@ -2357,19 +2357,19 @@
         <v>5</v>
       </c>
       <c r="I35">
-        <v>41250</v>
+        <v>45375</v>
       </c>
       <c r="J35">
-        <v>82500</v>
+        <v>90750</v>
       </c>
       <c r="K35">
-        <v>16500</v>
+        <v>18150</v>
       </c>
       <c r="L35">
-        <v>24750</v>
+        <v>27225</v>
       </c>
       <c r="M35">
-        <v>165000</v>
+        <v>181500</v>
       </c>
       <c r="N35">
         <v>0.3</v>
@@ -2404,19 +2404,19 @@
         <v>5</v>
       </c>
       <c r="I36">
-        <v>33750</v>
+        <v>37125</v>
       </c>
       <c r="J36">
-        <v>67500</v>
+        <v>74250</v>
       </c>
       <c r="K36">
-        <v>13500</v>
+        <v>14850</v>
       </c>
       <c r="L36">
-        <v>20250</v>
+        <v>22275</v>
       </c>
       <c r="M36">
-        <v>135000</v>
+        <v>148500</v>
       </c>
       <c r="N36">
         <v>0.2</v>
@@ -2451,19 +2451,19 @@
         <v>5</v>
       </c>
       <c r="I37">
-        <v>36250</v>
+        <v>39875</v>
       </c>
       <c r="J37">
-        <v>72500</v>
+        <v>79750</v>
       </c>
       <c r="K37">
-        <v>14500</v>
+        <v>15950</v>
       </c>
       <c r="L37">
-        <v>21750</v>
+        <v>23925</v>
       </c>
       <c r="M37">
-        <v>145000</v>
+        <v>159500</v>
       </c>
       <c r="N37">
         <v>0.2</v>
@@ -2498,19 +2498,19 @@
         <v>5</v>
       </c>
       <c r="I38">
-        <v>41250</v>
+        <v>45375</v>
       </c>
       <c r="J38">
-        <v>82500</v>
+        <v>90750</v>
       </c>
       <c r="K38">
-        <v>16500</v>
+        <v>18150</v>
       </c>
       <c r="L38">
-        <v>24750</v>
+        <v>27225</v>
       </c>
       <c r="M38">
-        <v>165000</v>
+        <v>181500</v>
       </c>
       <c r="N38">
         <v>0.2</v>
@@ -2545,19 +2545,19 @@
         <v>5</v>
       </c>
       <c r="I39">
-        <v>43750</v>
+        <v>48125</v>
       </c>
       <c r="J39">
-        <v>87500</v>
+        <v>96250</v>
       </c>
       <c r="K39">
-        <v>17500</v>
+        <v>19250</v>
       </c>
       <c r="L39">
-        <v>26250</v>
+        <v>28875</v>
       </c>
       <c r="M39">
-        <v>175000</v>
+        <v>192500</v>
       </c>
       <c r="N39">
         <v>0.2</v>
@@ -2592,19 +2592,19 @@
         <v>5</v>
       </c>
       <c r="I40">
-        <v>41250</v>
+        <v>45375</v>
       </c>
       <c r="J40">
-        <v>82500</v>
+        <v>90750</v>
       </c>
       <c r="K40">
-        <v>16500</v>
+        <v>18150</v>
       </c>
       <c r="L40">
-        <v>24750</v>
+        <v>27225</v>
       </c>
       <c r="M40">
-        <v>165000</v>
+        <v>181500</v>
       </c>
       <c r="N40">
         <v>0.2</v>
@@ -2639,19 +2639,19 @@
         <v>5</v>
       </c>
       <c r="I41">
-        <v>43750</v>
+        <v>48125</v>
       </c>
       <c r="J41">
-        <v>87500</v>
+        <v>96250</v>
       </c>
       <c r="K41">
-        <v>17500</v>
+        <v>19250</v>
       </c>
       <c r="L41">
-        <v>26250</v>
+        <v>28875</v>
       </c>
       <c r="M41">
-        <v>175000</v>
+        <v>192500</v>
       </c>
       <c r="N41">
         <v>0.2</v>
@@ -2686,19 +2686,19 @@
         <v>5</v>
       </c>
       <c r="I42">
-        <v>41250</v>
+        <v>45375</v>
       </c>
       <c r="J42">
-        <v>82500</v>
+        <v>90750</v>
       </c>
       <c r="K42">
-        <v>16500</v>
+        <v>18150</v>
       </c>
       <c r="L42">
-        <v>24750</v>
+        <v>27225</v>
       </c>
       <c r="M42">
-        <v>165000</v>
+        <v>181500</v>
       </c>
       <c r="N42">
         <v>0.2</v>
@@ -2733,19 +2733,19 @@
         <v>5</v>
       </c>
       <c r="I43">
-        <v>43750</v>
+        <v>48125</v>
       </c>
       <c r="J43">
-        <v>87500</v>
+        <v>96250</v>
       </c>
       <c r="K43">
-        <v>17500</v>
+        <v>19250</v>
       </c>
       <c r="L43">
-        <v>26250</v>
+        <v>28875</v>
       </c>
       <c r="M43">
-        <v>175000</v>
+        <v>192500</v>
       </c>
       <c r="N43">
         <v>0.2</v>
@@ -2780,19 +2780,19 @@
         <v>5</v>
       </c>
       <c r="I44">
-        <v>41250</v>
+        <v>45375</v>
       </c>
       <c r="J44">
-        <v>82500</v>
+        <v>90750</v>
       </c>
       <c r="K44">
-        <v>16500</v>
+        <v>18150</v>
       </c>
       <c r="L44">
-        <v>24750</v>
+        <v>27225</v>
       </c>
       <c r="M44">
-        <v>165000</v>
+        <v>181500</v>
       </c>
       <c r="N44">
         <v>0.2</v>
@@ -2827,19 +2827,19 @@
         <v>5</v>
       </c>
       <c r="I45">
-        <v>43750</v>
+        <v>48125</v>
       </c>
       <c r="J45">
-        <v>87500</v>
+        <v>96250</v>
       </c>
       <c r="K45">
-        <v>17500</v>
+        <v>19250</v>
       </c>
       <c r="L45">
-        <v>26250</v>
+        <v>28875</v>
       </c>
       <c r="M45">
-        <v>175000</v>
+        <v>192500</v>
       </c>
       <c r="N45">
         <v>0.2</v>
@@ -2874,19 +2874,19 @@
         <v>5</v>
       </c>
       <c r="I46">
-        <v>41250</v>
+        <v>45375</v>
       </c>
       <c r="J46">
-        <v>82500</v>
+        <v>90750</v>
       </c>
       <c r="K46">
-        <v>16500</v>
+        <v>18150</v>
       </c>
       <c r="L46">
-        <v>24750</v>
+        <v>27225</v>
       </c>
       <c r="M46">
-        <v>165000</v>
+        <v>181500</v>
       </c>
       <c r="N46">
         <v>0.2</v>
@@ -2921,19 +2921,19 @@
         <v>5</v>
       </c>
       <c r="I47">
-        <v>43750</v>
+        <v>48125</v>
       </c>
       <c r="J47">
-        <v>87500</v>
+        <v>96250</v>
       </c>
       <c r="K47">
-        <v>17500</v>
+        <v>19250</v>
       </c>
       <c r="L47">
-        <v>26250</v>
+        <v>28875</v>
       </c>
       <c r="M47">
-        <v>175000</v>
+        <v>192500</v>
       </c>
       <c r="N47">
         <v>0.2</v>
@@ -2968,19 +2968,19 @@
         <v>5</v>
       </c>
       <c r="I48">
-        <v>41250</v>
+        <v>45375</v>
       </c>
       <c r="J48">
-        <v>82500</v>
+        <v>90750</v>
       </c>
       <c r="K48">
-        <v>16500</v>
+        <v>18150</v>
       </c>
       <c r="L48">
-        <v>24750</v>
+        <v>27225</v>
       </c>
       <c r="M48">
-        <v>165000</v>
+        <v>181500</v>
       </c>
       <c r="N48">
         <v>0.3</v>
@@ -3015,19 +3015,19 @@
         <v>5</v>
       </c>
       <c r="I49">
-        <v>43750</v>
+        <v>48125</v>
       </c>
       <c r="J49">
-        <v>87500</v>
+        <v>96250</v>
       </c>
       <c r="K49">
-        <v>17500</v>
+        <v>19250</v>
       </c>
       <c r="L49">
-        <v>26250</v>
+        <v>28875</v>
       </c>
       <c r="M49">
-        <v>175000</v>
+        <v>192500</v>
       </c>
       <c r="N49">
         <v>0.3</v>
@@ -3062,19 +3062,19 @@
         <v>5</v>
       </c>
       <c r="I50">
-        <v>41250</v>
+        <v>45375</v>
       </c>
       <c r="J50">
-        <v>82500</v>
+        <v>90750</v>
       </c>
       <c r="K50">
-        <v>16500</v>
+        <v>18150</v>
       </c>
       <c r="L50">
-        <v>24750</v>
+        <v>27225</v>
       </c>
       <c r="M50">
-        <v>165000</v>
+        <v>181500</v>
       </c>
       <c r="N50">
         <v>0.3</v>
@@ -3109,19 +3109,19 @@
         <v>5</v>
       </c>
       <c r="I51">
-        <v>43750</v>
+        <v>48125</v>
       </c>
       <c r="J51">
-        <v>87500</v>
+        <v>96250</v>
       </c>
       <c r="K51">
-        <v>17500</v>
+        <v>19250</v>
       </c>
       <c r="L51">
-        <v>26250</v>
+        <v>28875</v>
       </c>
       <c r="M51">
-        <v>175000</v>
+        <v>192500</v>
       </c>
       <c r="N51">
         <v>0.3</v>
@@ -3156,19 +3156,19 @@
         <v>5</v>
       </c>
       <c r="I52">
-        <v>45000</v>
+        <v>49500</v>
       </c>
       <c r="J52">
-        <v>90000</v>
+        <v>99000</v>
       </c>
       <c r="K52">
-        <v>18000</v>
+        <v>19800</v>
       </c>
       <c r="L52">
-        <v>27000</v>
+        <v>29700</v>
       </c>
       <c r="M52">
-        <v>180000</v>
+        <v>198000</v>
       </c>
       <c r="N52">
         <v>0.3</v>
@@ -3203,19 +3203,19 @@
         <v>5</v>
       </c>
       <c r="I53">
-        <v>37500</v>
+        <v>41250</v>
       </c>
       <c r="J53">
-        <v>75000</v>
+        <v>82500</v>
       </c>
       <c r="K53">
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="L53">
-        <v>22500</v>
+        <v>24750</v>
       </c>
       <c r="M53">
-        <v>150000</v>
+        <v>165000</v>
       </c>
       <c r="N53">
         <v>0.2</v>
@@ -3250,19 +3250,19 @@
         <v>5</v>
       </c>
       <c r="I54">
-        <v>40000</v>
+        <v>44000</v>
       </c>
       <c r="J54">
-        <v>80000</v>
+        <v>88000</v>
       </c>
       <c r="K54">
-        <v>16000</v>
+        <v>17600</v>
       </c>
       <c r="L54">
-        <v>24000</v>
+        <v>26400</v>
       </c>
       <c r="M54">
-        <v>160000</v>
+        <v>176000</v>
       </c>
       <c r="N54">
         <v>0.2</v>
@@ -3297,19 +3297,19 @@
         <v>5</v>
       </c>
       <c r="I55">
-        <v>45000</v>
+        <v>49500</v>
       </c>
       <c r="J55">
-        <v>90000</v>
+        <v>99000</v>
       </c>
       <c r="K55">
-        <v>18000</v>
+        <v>19800</v>
       </c>
       <c r="L55">
-        <v>27000</v>
+        <v>29700</v>
       </c>
       <c r="M55">
-        <v>180000</v>
+        <v>198000</v>
       </c>
       <c r="N55">
         <v>0.2</v>
@@ -3344,19 +3344,19 @@
         <v>5</v>
       </c>
       <c r="I56">
-        <v>47500</v>
+        <v>52250</v>
       </c>
       <c r="J56">
-        <v>95000</v>
+        <v>104500</v>
       </c>
       <c r="K56">
-        <v>19000</v>
+        <v>20900</v>
       </c>
       <c r="L56">
-        <v>28500</v>
+        <v>31350</v>
       </c>
       <c r="M56">
-        <v>190000</v>
+        <v>209000</v>
       </c>
       <c r="N56">
         <v>0.2</v>
@@ -3391,19 +3391,19 @@
         <v>5</v>
       </c>
       <c r="I57">
-        <v>45000</v>
+        <v>49500</v>
       </c>
       <c r="J57">
-        <v>90000</v>
+        <v>99000</v>
       </c>
       <c r="K57">
-        <v>18000</v>
+        <v>19800</v>
       </c>
       <c r="L57">
-        <v>27000</v>
+        <v>29700</v>
       </c>
       <c r="M57">
-        <v>180000</v>
+        <v>198000</v>
       </c>
       <c r="N57">
         <v>0.2</v>
@@ -3438,19 +3438,19 @@
         <v>5</v>
       </c>
       <c r="I58">
-        <v>47500</v>
+        <v>52250</v>
       </c>
       <c r="J58">
-        <v>95000</v>
+        <v>104500</v>
       </c>
       <c r="K58">
-        <v>19000</v>
+        <v>20900</v>
       </c>
       <c r="L58">
-        <v>28500</v>
+        <v>31350</v>
       </c>
       <c r="M58">
-        <v>190000</v>
+        <v>209000</v>
       </c>
       <c r="N58">
         <v>0.2</v>
@@ -3485,19 +3485,19 @@
         <v>5</v>
       </c>
       <c r="I59">
-        <v>45000</v>
+        <v>49500</v>
       </c>
       <c r="J59">
-        <v>90000</v>
+        <v>99000</v>
       </c>
       <c r="K59">
-        <v>18000</v>
+        <v>19800</v>
       </c>
       <c r="L59">
-        <v>27000</v>
+        <v>29700</v>
       </c>
       <c r="M59">
-        <v>180000</v>
+        <v>198000</v>
       </c>
       <c r="N59">
         <v>0.2</v>
@@ -3532,19 +3532,19 @@
         <v>5</v>
       </c>
       <c r="I60">
-        <v>47500</v>
+        <v>52250</v>
       </c>
       <c r="J60">
-        <v>95000</v>
+        <v>104500</v>
       </c>
       <c r="K60">
-        <v>19000</v>
+        <v>20900</v>
       </c>
       <c r="L60">
-        <v>28500</v>
+        <v>31350</v>
       </c>
       <c r="M60">
-        <v>190000</v>
+        <v>209000</v>
       </c>
       <c r="N60">
         <v>0.2</v>
@@ -3579,19 +3579,19 @@
         <v>5</v>
       </c>
       <c r="I61">
-        <v>45000</v>
+        <v>49500</v>
       </c>
       <c r="J61">
-        <v>90000</v>
+        <v>99000</v>
       </c>
       <c r="K61">
-        <v>18000</v>
+        <v>19800</v>
       </c>
       <c r="L61">
-        <v>27000</v>
+        <v>29700</v>
       </c>
       <c r="M61">
-        <v>180000</v>
+        <v>198000</v>
       </c>
       <c r="N61">
         <v>0.2</v>
@@ -3626,19 +3626,19 @@
         <v>5</v>
       </c>
       <c r="I62">
-        <v>47500</v>
+        <v>52250</v>
       </c>
       <c r="J62">
-        <v>95000</v>
+        <v>104500</v>
       </c>
       <c r="K62">
-        <v>19000</v>
+        <v>20900</v>
       </c>
       <c r="L62">
-        <v>28500</v>
+        <v>31350</v>
       </c>
       <c r="M62">
-        <v>190000</v>
+        <v>209000</v>
       </c>
       <c r="N62">
         <v>0.2</v>
@@ -3673,19 +3673,19 @@
         <v>5</v>
       </c>
       <c r="I63">
-        <v>45000</v>
+        <v>49500</v>
       </c>
       <c r="J63">
-        <v>90000</v>
+        <v>99000</v>
       </c>
       <c r="K63">
-        <v>18000</v>
+        <v>19800</v>
       </c>
       <c r="L63">
-        <v>27000</v>
+        <v>29700</v>
       </c>
       <c r="M63">
-        <v>180000</v>
+        <v>198000</v>
       </c>
       <c r="N63">
         <v>0.2</v>
@@ -3720,19 +3720,19 @@
         <v>5</v>
       </c>
       <c r="I64">
-        <v>47500</v>
+        <v>52250</v>
       </c>
       <c r="J64">
-        <v>95000</v>
+        <v>104500</v>
       </c>
       <c r="K64">
-        <v>19000</v>
+        <v>20900</v>
       </c>
       <c r="L64">
-        <v>28500</v>
+        <v>31350</v>
       </c>
       <c r="M64">
-        <v>190000</v>
+        <v>209000</v>
       </c>
       <c r="N64">
         <v>0.2</v>
@@ -3767,19 +3767,19 @@
         <v>5</v>
       </c>
       <c r="I65">
-        <v>45000</v>
+        <v>49500</v>
       </c>
       <c r="J65">
-        <v>90000</v>
+        <v>99000</v>
       </c>
       <c r="K65">
-        <v>18000</v>
+        <v>19800</v>
       </c>
       <c r="L65">
-        <v>27000</v>
+        <v>29700</v>
       </c>
       <c r="M65">
-        <v>180000</v>
+        <v>198000</v>
       </c>
       <c r="N65">
         <v>0.3</v>
@@ -3814,19 +3814,19 @@
         <v>5</v>
       </c>
       <c r="I66">
-        <v>47500</v>
+        <v>52250</v>
       </c>
       <c r="J66">
-        <v>95000</v>
+        <v>104500</v>
       </c>
       <c r="K66">
-        <v>19000</v>
+        <v>20900</v>
       </c>
       <c r="L66">
-        <v>28500</v>
+        <v>31350</v>
       </c>
       <c r="M66">
-        <v>190000</v>
+        <v>209000</v>
       </c>
       <c r="N66">
         <v>0.3</v>
@@ -3861,19 +3861,19 @@
         <v>5</v>
       </c>
       <c r="I67">
-        <v>45000</v>
+        <v>49500</v>
       </c>
       <c r="J67">
-        <v>90000</v>
+        <v>99000</v>
       </c>
       <c r="K67">
-        <v>18000</v>
+        <v>19800</v>
       </c>
       <c r="L67">
-        <v>27000</v>
+        <v>29700</v>
       </c>
       <c r="M67">
-        <v>180000</v>
+        <v>198000</v>
       </c>
       <c r="N67">
         <v>0.3</v>
@@ -3908,19 +3908,19 @@
         <v>5</v>
       </c>
       <c r="I68">
-        <v>47500</v>
+        <v>52250</v>
       </c>
       <c r="J68">
-        <v>95000</v>
+        <v>104500</v>
       </c>
       <c r="K68">
-        <v>19000</v>
+        <v>20900</v>
       </c>
       <c r="L68">
-        <v>28500</v>
+        <v>31350</v>
       </c>
       <c r="M68">
-        <v>190000</v>
+        <v>209000</v>
       </c>
       <c r="N68">
         <v>0.3</v>
@@ -3955,19 +3955,19 @@
         <v>5</v>
       </c>
       <c r="I69">
-        <v>48750</v>
+        <v>53625</v>
       </c>
       <c r="J69">
-        <v>97500</v>
+        <v>107250</v>
       </c>
       <c r="K69">
-        <v>19500</v>
+        <v>21450</v>
       </c>
       <c r="L69">
-        <v>29250</v>
+        <v>32175</v>
       </c>
       <c r="M69">
-        <v>195000</v>
+        <v>214500</v>
       </c>
       <c r="N69">
         <v>0.3</v>
@@ -4002,19 +4002,19 @@
         <v>5</v>
       </c>
       <c r="I70">
-        <v>41250</v>
+        <v>45375</v>
       </c>
       <c r="J70">
-        <v>82500</v>
+        <v>90750</v>
       </c>
       <c r="K70">
-        <v>16500</v>
+        <v>18150</v>
       </c>
       <c r="L70">
-        <v>24750</v>
+        <v>27225</v>
       </c>
       <c r="M70">
-        <v>165000</v>
+        <v>181500</v>
       </c>
       <c r="N70">
         <v>0.2</v>
@@ -4049,19 +4049,19 @@
         <v>5</v>
       </c>
       <c r="I71">
-        <v>43750</v>
+        <v>48125</v>
       </c>
       <c r="J71">
-        <v>87500</v>
+        <v>96250</v>
       </c>
       <c r="K71">
-        <v>17500</v>
+        <v>19250</v>
       </c>
       <c r="L71">
-        <v>26250</v>
+        <v>28875</v>
       </c>
       <c r="M71">
-        <v>175000</v>
+        <v>192500</v>
       </c>
       <c r="N71">
         <v>0.2</v>
@@ -4095,20 +4095,8 @@
       <c r="H72">
         <v>1.3</v>
       </c>
-      <c r="I72">
-        <v>4000</v>
-      </c>
-      <c r="J72">
-        <v>8000</v>
-      </c>
-      <c r="K72">
-        <v>1500</v>
-      </c>
-      <c r="L72">
-        <v>1500</v>
-      </c>
       <c r="M72">
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="N72">
         <v>0.3</v>

</xml_diff>